<commit_message>
WIP: local changes before pull
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/安全体检报告/风险清单/弱口令清单.xlsx
+++ b/安全体检报告/风险清单/弱口令清单.xlsx
@@ -653,7 +653,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -740,7 +740,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -922,7 +922,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1017,7 +1017,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1104,7 +1104,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1191,7 +1191,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1282,7 +1282,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1373,7 +1373,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1460,7 +1460,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1634,7 +1634,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>192.168.79.242</t>
+          <t>192.168.75.50</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1990,7 +1990,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>192.168.73.179</t>
+          <t>192.168.79.242</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2077,7 +2077,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>192.168.75.50</t>
+          <t>192.168.73.179</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>192.168.79.242</t>
+          <t>192.168.79.227</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2251,7 +2251,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>192.168.75.50</t>
+          <t>192.168.79.227</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2338,7 +2338,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>192.168.73.179</t>
+          <t>192.168.75.50</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>192.168.79.227</t>
+          <t>192.168.73.179</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>192.168.79.227</t>
+          <t>192.168.79.242</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2599,7 +2599,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2690,7 +2690,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>192.168.75.187</t>
+          <t>192.168.76.68</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>192.168.76.68</t>
+          <t>192.168.75.187</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>192.168.73.182</t>
+          <t>192.168.75.187</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3247,7 +3247,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>192.168.75.187</t>
+          <t>192.168.73.182</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>192.168.74.62</t>
+          <t>192.168.71.140</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3477,7 +3477,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3508,7 +3508,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>192.168.74.62</t>
+          <t>192.168.78.80</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3564,7 +3564,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3682,7 +3682,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>192.168.75.136</t>
+          <t>192.168.76.106</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3943,7 +3943,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>192.168.76.106</t>
+          <t>192.168.75.136</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4030,7 +4030,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>192.168.71.140</t>
+          <t>192.168.74.62</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4117,7 +4117,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>192.168.78.80</t>
+          <t>192.168.74.62</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4173,7 +4173,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4260,7 +4260,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -4347,7 +4347,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4434,7 +4434,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -4521,7 +4521,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -4608,7 +4608,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -4695,7 +4695,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -4782,7 +4782,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -4869,7 +4869,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -4956,7 +4956,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -5130,7 +5130,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -5161,7 +5161,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>192.168.75.224</t>
+          <t>192.168.74.169</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5304,7 +5304,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -5335,7 +5335,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>192.168.74.169</t>
+          <t>192.168.75.224</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -5478,7 +5478,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -5509,7 +5509,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>192.168.79.137</t>
+          <t>192.168.79.44</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -5565,7 +5565,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -5596,7 +5596,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>192.168.79.137</t>
+          <t>192.168.78.215</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5739,7 +5739,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -5770,7 +5770,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>192.168.78.215</t>
+          <t>192.168.79.137</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -5826,7 +5826,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -5857,7 +5857,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>192.168.79.44</t>
+          <t>192.168.79.137</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5913,7 +5913,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -6000,7 +6000,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -6087,7 +6087,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -6118,7 +6118,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>192.168.75.79</t>
+          <t>192.168.75.46</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -6348,7 +6348,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -6379,7 +6379,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>192.168.75.46</t>
+          <t>192.168.75.79</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -6435,7 +6435,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -6522,7 +6522,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -6609,7 +6609,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -6696,7 +6696,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -6901,7 +6901,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>192.168.72.113</t>
+          <t>192.168.72.42</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -7075,7 +7075,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>192.168.72.42</t>
+          <t>192.168.72.113</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -7131,7 +7131,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -7162,7 +7162,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>192.168.73.85</t>
+          <t>192.168.70.3</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -7249,7 +7249,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>192.168.77.110</t>
+          <t>192.168.70.3</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -7336,7 +7336,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>192.168.70.3</t>
+          <t>192.168.77.110</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -7392,7 +7392,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -7423,7 +7423,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>192.168.70.3</t>
+          <t>192.168.73.85</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -7510,7 +7510,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>192.168.73.85</t>
+          <t>192.168.77.110</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -7597,7 +7597,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>192.168.77.110</t>
+          <t>192.168.73.85</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -7653,7 +7653,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -7740,7 +7740,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -7827,7 +7827,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -7918,7 +7918,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>192.168.74.124</t>
+          <t>192.168.75.103</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>192.168.75.103</t>
+          <t>192.168.74.124</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -8475,7 +8475,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>192.168.74.124</t>
+          <t>192.168.75.103</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -8562,7 +8562,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>192.168.75.103</t>
+          <t>192.168.74.124</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -8705,7 +8705,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -8823,7 +8823,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>192.168.71.61</t>
+          <t>192.168.71.200</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -8910,7 +8910,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>192.168.71.200</t>
+          <t>192.168.71.61</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -8966,7 +8966,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -9053,7 +9053,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -9084,7 +9084,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>192.168.78.28</t>
+          <t>192.168.77.15</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -9171,7 +9171,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>192.168.71.200</t>
+          <t>192.168.77.15</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -9227,7 +9227,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -9258,7 +9258,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>192.168.78.28</t>
+          <t>192.168.71.61</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -9314,7 +9314,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -9345,7 +9345,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>192.168.71.61</t>
+          <t>192.168.78.28</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -9432,7 +9432,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>192.168.77.15</t>
+          <t>192.168.71.200</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -9488,7 +9488,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -9519,7 +9519,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>192.168.77.15</t>
+          <t>192.168.78.28</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -9693,7 +9693,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>192.168.74.36</t>
+          <t>192.168.71.234</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -9867,7 +9867,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>192.168.71.234</t>
+          <t>192.168.74.36</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -9923,7 +9923,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -10010,7 +10010,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -10097,7 +10097,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -10184,7 +10184,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -10445,7 +10445,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -10532,7 +10532,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -10793,7 +10793,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -10880,7 +10880,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -11054,7 +11054,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -11141,7 +11141,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -11228,7 +11228,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -11758,7 +11758,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -11932,7 +11932,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -12019,7 +12019,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -12050,7 +12050,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>192.168.75.222</t>
+          <t>192.168.72.30</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -12137,7 +12137,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>192.168.72.30</t>
+          <t>192.168.75.222</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -12193,7 +12193,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -12367,7 +12367,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -12454,7 +12454,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -12541,7 +12541,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>192.168.76.235</t>
+          <t>192.168.78.251</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -12628,7 +12628,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -12659,7 +12659,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>192.168.78.251</t>
+          <t>192.168.76.235</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -12715,7 +12715,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -12746,7 +12746,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>192.168.76.235</t>
+          <t>192.168.78.251</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -12802,7 +12802,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -12833,7 +12833,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>192.168.78.251</t>
+          <t>192.168.76.235</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -12889,7 +12889,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -12976,7 +12976,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -13063,7 +13063,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -13150,7 +13150,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -13585,7 +13585,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -13672,7 +13672,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -13790,7 +13790,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>192.168.77.11</t>
+          <t>192.168.70.247</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -13964,7 +13964,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>192.168.70.247</t>
+          <t>192.168.77.11</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -14281,7 +14281,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -14312,7 +14312,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>192.168.77.80</t>
+          <t>192.168.75.153</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -14368,7 +14368,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -14399,7 +14399,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>192.168.75.153</t>
+          <t>192.168.77.80</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -14455,7 +14455,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -14486,7 +14486,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>192.168.77.80</t>
+          <t>192.168.75.153</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -14542,7 +14542,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -14573,7 +14573,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>192.168.75.153</t>
+          <t>192.168.77.80</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -14803,7 +14803,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -14890,7 +14890,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -14977,7 +14977,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -15008,7 +15008,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>192.168.76.131</t>
+          <t>192.168.74.81</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -15064,7 +15064,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -15095,7 +15095,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>192.168.74.236</t>
+          <t>192.168.71.100</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -15151,7 +15151,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -15182,7 +15182,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>192.168.77.91</t>
+          <t>192.168.78.110</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -15269,7 +15269,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>192.168.74.81</t>
+          <t>192.168.75.249</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>192.168.76.131</t>
+          <t>192.168.72.128</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -15443,7 +15443,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>192.168.72.128</t>
+          <t>192.168.76.131</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -15530,7 +15530,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>192.168.75.249</t>
+          <t>192.168.74.81</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -15586,7 +15586,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -15617,7 +15617,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>192.168.71.100</t>
+          <t>192.168.77.91</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -15704,7 +15704,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>192.168.78.110</t>
+          <t>192.168.76.131</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -15791,7 +15791,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>192.168.74.81</t>
+          <t>192.168.74.236</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -15847,7 +15847,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -15878,7 +15878,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>192.168.74.236</t>
+          <t>192.168.79.136</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -15934,7 +15934,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -15965,7 +15965,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>192.168.75.249</t>
+          <t>192.168.79.136</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -16021,7 +16021,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -16052,7 +16052,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>192.168.72.128</t>
+          <t>192.168.78.110</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -16108,7 +16108,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -16139,7 +16139,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>192.168.79.185</t>
+          <t>192.168.72.98</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -16226,7 +16226,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>192.168.77.91</t>
+          <t>192.168.73.206</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -16313,7 +16313,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>192.168.79.185</t>
+          <t>192.168.71.100</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -16369,7 +16369,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -16487,7 +16487,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>192.168.79.136</t>
+          <t>192.168.72.98</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -16574,7 +16574,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>192.168.71.100</t>
+          <t>192.168.79.185</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -16661,7 +16661,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>192.168.72.98</t>
+          <t>192.168.77.91</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -16717,7 +16717,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -16748,7 +16748,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>192.168.73.206</t>
+          <t>192.168.72.128</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -16804,7 +16804,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -16835,7 +16835,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>192.168.78.110</t>
+          <t>192.168.79.185</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -16891,7 +16891,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -16922,7 +16922,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>192.168.79.136</t>
+          <t>192.168.74.236</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -17009,7 +17009,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>192.168.72.98</t>
+          <t>192.168.75.249</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -17239,7 +17239,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -17270,7 +17270,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>192.168.74.195</t>
+          <t>192.168.72.229</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -17413,7 +17413,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -17444,7 +17444,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>192.168.72.229</t>
+          <t>192.168.74.195</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -17587,7 +17587,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -17674,7 +17674,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -18140,7 +18140,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>192.168.78.76</t>
+          <t>192.168.73.123</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -18196,7 +18196,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -18227,7 +18227,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>192.168.73.54</t>
+          <t>192.168.78.159</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -18314,7 +18314,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>192.168.73.123</t>
+          <t>192.168.74.216</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -18370,7 +18370,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -18401,7 +18401,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>192.168.73.54</t>
+          <t>192.168.76.133</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -18488,7 +18488,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>192.168.72.210</t>
+          <t>192.168.75.177</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -18544,7 +18544,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -18575,7 +18575,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>192.168.78.76</t>
+          <t>192.168.70.81</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -18662,7 +18662,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>192.168.71.153</t>
+          <t>192.168.78.159</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -18718,7 +18718,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -18749,7 +18749,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>192.168.70.149</t>
+          <t>192.168.71.153</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -18805,7 +18805,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -18836,7 +18836,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>192.168.78.159</t>
+          <t>192.168.70.149</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -18892,7 +18892,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -18923,7 +18923,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>192.168.70.81</t>
+          <t>192.168.78.76</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
@@ -19010,7 +19010,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>192.168.75.177</t>
+          <t>192.168.72.210</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
@@ -19097,7 +19097,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>192.168.78.159</t>
+          <t>192.168.73.54</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -19184,7 +19184,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>192.168.76.133</t>
+          <t>192.168.73.123</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
@@ -19271,7 +19271,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>192.168.74.216</t>
+          <t>192.168.78.76</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -19327,7 +19327,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -19358,7 +19358,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>192.168.73.123</t>
+          <t>192.168.73.54</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -19414,7 +19414,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -19445,7 +19445,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>192.168.72.210</t>
+          <t>192.168.75.219</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -19532,7 +19532,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>192.168.71.153</t>
+          <t>192.168.76.133</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -19619,7 +19619,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>192.168.70.81</t>
+          <t>192.168.70.149</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
@@ -19675,7 +19675,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -19706,7 +19706,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>192.168.72.162</t>
+          <t>192.168.75.177</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
@@ -19793,7 +19793,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>192.168.74.216</t>
+          <t>192.168.72.162</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
@@ -19936,7 +19936,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -20054,7 +20054,7 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>192.168.75.177</t>
+          <t>192.168.70.81</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -20141,7 +20141,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>192.168.76.133</t>
+          <t>192.168.74.216</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -20197,7 +20197,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -20228,7 +20228,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>192.168.75.219</t>
+          <t>192.168.72.210</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -20284,7 +20284,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -20315,7 +20315,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>192.168.70.149</t>
+          <t>192.168.71.153</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -20402,7 +20402,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>192.168.74.201</t>
+          <t>192.168.71.162</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
@@ -20489,7 +20489,7 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>192.168.79.115</t>
+          <t>192.168.72.133</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
@@ -20545,7 +20545,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -20632,7 +20632,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -20663,7 +20663,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>192.168.79.115</t>
+          <t>192.168.78.36</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -20750,7 +20750,7 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>192.168.75.22</t>
+          <t>192.168.71.162</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
@@ -20806,7 +20806,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -20837,7 +20837,7 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>192.168.79.14</t>
+          <t>192.168.74.166</t>
         </is>
       </c>
       <c r="I234" t="inlineStr">
@@ -20924,7 +20924,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>192.168.72.133</t>
+          <t>192.168.75.22</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -20980,7 +20980,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -21011,7 +21011,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>192.168.74.166</t>
+          <t>192.168.79.14</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -21098,7 +21098,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>192.168.71.162</t>
+          <t>192.168.72.133</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
@@ -21154,7 +21154,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -21185,7 +21185,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>192.168.72.133</t>
+          <t>192.168.74.201</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
@@ -21272,7 +21272,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>192.168.75.15</t>
+          <t>192.168.79.115</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -21359,7 +21359,7 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>192.168.78.36</t>
+          <t>192.168.75.15</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
@@ -21446,7 +21446,7 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>192.168.71.162</t>
+          <t>192.168.79.115</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
@@ -21533,7 +21533,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>192.168.72.14</t>
+          <t>192.168.74.201</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
@@ -21589,7 +21589,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -21620,7 +21620,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>192.168.78.36</t>
+          <t>192.168.74.136</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
@@ -21676,7 +21676,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -21707,7 +21707,7 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>192.168.72.14</t>
+          <t>192.168.79.14</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
@@ -21794,7 +21794,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>192.168.74.155</t>
+          <t>192.168.74.136</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
@@ -21881,7 +21881,7 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>192.168.74.155</t>
+          <t>192.168.75.22</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
@@ -22024,7 +22024,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -22055,7 +22055,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>192.168.75.22</t>
+          <t>192.168.74.155</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -22142,7 +22142,7 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>192.168.74.201</t>
+          <t>192.168.78.36</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
@@ -22229,7 +22229,7 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>192.168.79.14</t>
+          <t>192.168.74.155</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
@@ -22316,7 +22316,7 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>192.168.74.136</t>
+          <t>192.168.72.14</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
@@ -22403,7 +22403,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>192.168.74.136</t>
+          <t>192.168.72.14</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -22807,7 +22807,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -22894,7 +22894,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -23155,7 +23155,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -23242,7 +23242,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -23329,7 +23329,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Redis 弱密码</t>
+          <t>SSH 弱密码</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -23416,7 +23416,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>SSH 弱密码</t>
+          <t>Redis 弱密码</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -23708,7 +23708,7 @@
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>192.168.54.68</t>
+          <t>192.168.51.66</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
@@ -23723,7 +23723,7 @@
       </c>
       <c r="K267" t="inlineStr">
         <is>
-          <t>父组名</t>
+          <t>子组名</t>
         </is>
       </c>
       <c r="L267" t="inlineStr"/>
@@ -23799,7 +23799,7 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>192.168.51.66</t>
+          <t>192.168.54.68</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
@@ -23814,7 +23814,7 @@
       </c>
       <c r="K268" t="inlineStr">
         <is>
-          <t>子组名</t>
+          <t>父组名</t>
         </is>
       </c>
       <c r="L268" t="inlineStr"/>
@@ -23890,12 +23890,12 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>192.168.54.174</t>
+          <t>192.168.54.213</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
         <is>
-          <t>服务器</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="J269" t="inlineStr">
@@ -23916,7 +23916,7 @@
       </c>
       <c r="N269" t="inlineStr">
         <is>
-          <t>退库资产</t>
+          <t>台账资产</t>
         </is>
       </c>
       <c r="O269" t="inlineStr">
@@ -23981,12 +23981,12 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>192.168.54.213</t>
+          <t>192.168.54.174</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>服务器</t>
         </is>
       </c>
       <c r="J270" t="inlineStr">
@@ -24007,7 +24007,7 @@
       </c>
       <c r="N270" t="inlineStr">
         <is>
-          <t>台账资产</t>
+          <t>退库资产</t>
         </is>
       </c>
       <c r="O270" t="inlineStr">
@@ -24072,12 +24072,12 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>192.168.51.66</t>
+          <t>192.168.54.213</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>服务器</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="J271" t="inlineStr">
@@ -24087,7 +24087,7 @@
       </c>
       <c r="K271" t="inlineStr">
         <is>
-          <t>子组名</t>
+          <t>test1111</t>
         </is>
       </c>
       <c r="L271" t="inlineStr"/>
@@ -24098,7 +24098,7 @@
       </c>
       <c r="N271" t="inlineStr">
         <is>
-          <t>退库资产</t>
+          <t>台账资产</t>
         </is>
       </c>
       <c r="O271" t="inlineStr">
@@ -24163,7 +24163,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>192.168.54.174</t>
+          <t>192.168.54.68</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
@@ -24178,7 +24178,7 @@
       </c>
       <c r="K272" t="inlineStr">
         <is>
-          <t>test1111</t>
+          <t>父组名</t>
         </is>
       </c>
       <c r="L272" t="inlineStr"/>
@@ -24254,7 +24254,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>192.168.54.68</t>
+          <t>192.168.54.174</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -24269,7 +24269,7 @@
       </c>
       <c r="K273" t="inlineStr">
         <is>
-          <t>父组名</t>
+          <t>test1111</t>
         </is>
       </c>
       <c r="L273" t="inlineStr"/>
@@ -24345,12 +24345,12 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>192.168.54.213</t>
+          <t>192.168.51.66</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>服务器</t>
         </is>
       </c>
       <c r="J274" t="inlineStr">
@@ -24360,7 +24360,7 @@
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t>test1111</t>
+          <t>子组名</t>
         </is>
       </c>
       <c r="L274" t="inlineStr"/>
@@ -24371,7 +24371,7 @@
       </c>
       <c r="N274" t="inlineStr">
         <is>
-          <t>台账资产</t>
+          <t>退库资产</t>
         </is>
       </c>
       <c r="O274" t="inlineStr">

</xml_diff>